<commit_message>
Small edits to data cleaning
</commit_message>
<xml_diff>
--- a/SGP_CONFIG/EOCT/2018/2018 EOC Course Sequence.xlsx
+++ b/SGP_CONFIG/EOCT/2018/2018 EOC Course Sequence.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="27127"/>
   <workbookPr autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="39360" yWindow="1900" windowWidth="27600" windowHeight="16540"/>
+    <workbookView xWindow="38000" yWindow="1360" windowWidth="27600" windowHeight="16540"/>
   </bookViews>
   <sheets>
     <sheet name="Final List" sheetId="11" r:id="rId1"/>
@@ -167,7 +167,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -262,6 +262,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -343,11 +359,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -445,9 +465,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="8">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
+    <cellStyle name="Followed Hyperlink" xfId="5" builtinId="9" hidden="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9" hidden="1"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Hyperlink" xfId="4" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8" hidden="1"/>
     <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -719,7 +743,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1885,6 +1909,7 @@
     <row r="137" s="9" customFormat="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="0" OnePage="0" WScale="0"/>

</xml_diff>